<commit_message>
agregar filtro por fecha al panel FEMP
</commit_message>
<xml_diff>
--- a/inscritos.xlsx
+++ b/inscritos.xlsx
@@ -413,12 +413,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -532,6 +532,160 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Mariali</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>franciscoedward296@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Medicina Táctica</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>17/04/2026 16:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>vargas</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>franciscoedward296@gmail.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Rescate y Evacuación</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>17/04/2026 17:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>yoel</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>franciscoedward296@gmail.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Primeros Auxilios Básicos</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>17/04/2026 17:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>reny</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>franciscoedward296@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Prevención del Abuso Sexual Infantil</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>17/04/2026 17:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>oto</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>franciscoedward296@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Primeros Auxilios Psicológicos</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>17/04/2026 17:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>iander</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>franciscoedward296@gmail.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Manejo de Arma de Fuego</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>17/04/2026 18:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>guillen</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>franciscoedward296@gmail.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Análisis Superior</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>17/04/2026 18:43</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>